<commit_message>
Update S32K3 DS & RM
</commit_message>
<xml_diff>
--- a/S32K3/S32K3xx_part_number_dashboard.xlsx
+++ b/S32K3/S32K3xx_part_number_dashboard.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nxp1-my.sharepoint.com/personal/harpal_singh_nxp_com/Documents/computer_data_1Apr2024/A_Workspace/DS/K3/DS/Rev12/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nxp1-my.sharepoint.com/personal/yiling_zhang_nxp_com1/Documents/Work/PRODUCT MANAGEMENT 2024-25/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="8_{9187731B-B225-4F06-9277-C19420E82616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7542921-952E-46F9-9E5C-8561990A67E4}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="8_{9187731B-B225-4F06-9277-C19420E82616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11CBAA32-3B74-46F9-AED5-470386F32E85}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="S32K3 part number dashboard" sheetId="4" r:id="rId1"/>
@@ -23,14 +23,14 @@
   <definedNames>
     <definedName name="_100_MaxQFP_GMUC">#REF!</definedName>
     <definedName name="_48_QFN_GMUC">#REF!</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'S32K3 part number dashboard'!$A$2:$M$236</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'S32K3 part number dashboard'!$A$2:$M$264</definedName>
     <definedName name="DPConsolidatedGrossMarginkUSD">'[1]Data Processing'!$L$1295:$AD$1297</definedName>
     <definedName name="DPConsolidatedQuantity">'[1]Data Processing'!$L$948:$AD$950</definedName>
     <definedName name="DPConsolidatedSaleskUSD">'[1]Data Processing'!$L$1271:$AD$1273</definedName>
     <definedName name="Ethernet">[2]Data!$D$7:$D$9</definedName>
     <definedName name="Security">[2]Data!$C$7:$C$10</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3068" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3434" uniqueCount="354">
   <si>
     <t>Product</t>
   </si>
@@ -1013,6 +1013,105 @@
   </si>
   <si>
     <t>6MB</t>
+  </si>
+  <si>
+    <t>S32K312NHT0MLLST</t>
+  </si>
+  <si>
+    <t>100LQFP</t>
+  </si>
+  <si>
+    <t>S32K312NHT0VLLST</t>
+  </si>
+  <si>
+    <t>S32K312NHT0VLLSR</t>
+  </si>
+  <si>
+    <t>S32K312NHT0MLLSR</t>
+  </si>
+  <si>
+    <t>S32K314EHT1MLLST</t>
+  </si>
+  <si>
+    <t>S32K314EHT1VLLST</t>
+  </si>
+  <si>
+    <t>S32K314NHT1VLLST</t>
+  </si>
+  <si>
+    <t>S32K314NHT1MLLST</t>
+  </si>
+  <si>
+    <t>S32K314EHT1VLLSR</t>
+  </si>
+  <si>
+    <t>S32K314EHT1MLLSR</t>
+  </si>
+  <si>
+    <t>S32K314NHT1VLLSR</t>
+  </si>
+  <si>
+    <t>S32K314NHT1MLLSR</t>
+  </si>
+  <si>
+    <t>S32K324EHT1MLLST</t>
+  </si>
+  <si>
+    <t>S32K324EHT1VLLST</t>
+  </si>
+  <si>
+    <t>S32K324NHT1VLLST</t>
+  </si>
+  <si>
+    <t>S32K324NHT1MLLST</t>
+  </si>
+  <si>
+    <t>S32K324EHT1VLLSR</t>
+  </si>
+  <si>
+    <t>S32K324EHT1MLLSR</t>
+  </si>
+  <si>
+    <t>S32K324NHT1VLLSR</t>
+  </si>
+  <si>
+    <t>S32K324NHT1MLLSR</t>
+  </si>
+  <si>
+    <t>S32K344EHT1MLLST</t>
+  </si>
+  <si>
+    <t>S32K344EHT1VLLST</t>
+  </si>
+  <si>
+    <t>S32K344NHT1VLLST</t>
+  </si>
+  <si>
+    <t>S32K344NHT1MLLST</t>
+  </si>
+  <si>
+    <t>S32K344EHT1VLLSR</t>
+  </si>
+  <si>
+    <t>S32K344EHT1MLLSR</t>
+  </si>
+  <si>
+    <t>S32K344NHT1VLLSR</t>
+  </si>
+  <si>
+    <t>S32K344NHT1MLLSR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Added K312/K3x4 - 100LQFP part numbers </t>
+  </si>
+  <si>
+    <t xml:space="preserve">superset </t>
+  </si>
+  <si>
+    <t>superset</t>
+  </si>
+  <si>
+    <t>Updated Avalability colume to align with sample status on nxp web</t>
   </si>
 </sst>
 </file>
@@ -1551,26 +1650,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75745F4E-7D5E-4F38-AD53-8B00FD2DCD73}">
-  <dimension ref="A1:AG236"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AG264"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.85546875" style="5" customWidth="1"/>
+    <col min="1" max="1" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.81640625" style="5" customWidth="1"/>
     <col min="4" max="4" width="23" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.54296875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
-    <col min="8" max="8" width="37.42578125" customWidth="1"/>
-    <col min="9" max="9" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="37.453125" customWidth="1"/>
+    <col min="9" max="9" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.81640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.140625" style="9"/>
+    <col min="15" max="15" width="9.1796875" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" ht="51.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>257</v>
       </c>
@@ -1587,7 +1686,7 @@
       <c r="L1" s="13"/>
       <c r="M1" s="13"/>
     </row>
-    <row r="2" spans="1:33" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1629,7 +1728,7 @@
       </c>
       <c r="O2" s="9"/>
     </row>
-    <row r="3" spans="1:33" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1688,7 +1787,7 @@
       <c r="AF3" s="6"/>
       <c r="AG3" s="6"/>
     </row>
-    <row r="4" spans="1:33" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -1748,7 +1847,7 @@
       <c r="AF4" s="6"/>
       <c r="AG4" s="6"/>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1808,7 +1907,7 @@
       <c r="AF5" s="6"/>
       <c r="AG5" s="6"/>
     </row>
-    <row r="6" spans="1:33" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -1867,7 +1966,7 @@
       <c r="AF6" s="6"/>
       <c r="AG6" s="6"/>
     </row>
-    <row r="7" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1927,7 +2026,7 @@
       <c r="AF7" s="6"/>
       <c r="AG7" s="6"/>
     </row>
-    <row r="8" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -1987,7 +2086,7 @@
       <c r="AF8" s="6"/>
       <c r="AG8" s="6"/>
     </row>
-    <row r="9" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -2029,7 +2128,7 @@
       </c>
       <c r="P9" s="6"/>
     </row>
-    <row r="10" spans="1:33" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -2072,7 +2171,7 @@
       <c r="O10" s="10"/>
       <c r="P10" s="6"/>
     </row>
-    <row r="11" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -2115,7 +2214,7 @@
       <c r="O11" s="8"/>
       <c r="P11" s="6"/>
     </row>
-    <row r="12" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -2157,7 +2256,7 @@
       </c>
       <c r="P12" s="6"/>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>38</v>
       </c>
@@ -2200,7 +2299,7 @@
       <c r="O13" s="10"/>
       <c r="P13" s="6"/>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -2243,7 +2342,7 @@
       <c r="O14" s="8"/>
       <c r="P14" s="6"/>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>38</v>
       </c>
@@ -2285,7 +2384,7 @@
       </c>
       <c r="P15" s="6"/>
     </row>
-    <row r="16" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>38</v>
       </c>
@@ -2328,7 +2427,7 @@
       <c r="O16" s="10"/>
       <c r="P16" s="6"/>
     </row>
-    <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>38</v>
       </c>
@@ -2371,7 +2470,7 @@
       <c r="O17" s="8"/>
       <c r="P17" s="6"/>
     </row>
-    <row r="18" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>38</v>
       </c>
@@ -2413,7 +2512,7 @@
       </c>
       <c r="P18" s="6"/>
     </row>
-    <row r="19" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>38</v>
       </c>
@@ -2456,7 +2555,7 @@
       <c r="O19" s="10"/>
       <c r="P19" s="6"/>
     </row>
-    <row r="20" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>38</v>
       </c>
@@ -2499,7 +2598,7 @@
       <c r="O20" s="8"/>
       <c r="P20" s="6"/>
     </row>
-    <row r="21" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>38</v>
       </c>
@@ -2541,7 +2640,7 @@
       </c>
       <c r="P21" s="6"/>
     </row>
-    <row r="22" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>38</v>
       </c>
@@ -2584,7 +2683,7 @@
       <c r="O22" s="10"/>
       <c r="P22" s="6"/>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>50</v>
       </c>
@@ -2627,7 +2726,7 @@
       <c r="O23" s="8"/>
       <c r="P23" s="6"/>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>50</v>
       </c>
@@ -2669,7 +2768,7 @@
       </c>
       <c r="P24" s="6"/>
     </row>
-    <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>50</v>
       </c>
@@ -2712,7 +2811,7 @@
       <c r="O25" s="10"/>
       <c r="P25" s="6"/>
     </row>
-    <row r="26" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>50</v>
       </c>
@@ -2755,7 +2854,7 @@
       <c r="O26" s="8"/>
       <c r="P26" s="6"/>
     </row>
-    <row r="27" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>50</v>
       </c>
@@ -2797,7 +2896,7 @@
       </c>
       <c r="P27" s="6"/>
     </row>
-    <row r="28" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>50</v>
       </c>
@@ -2840,7 +2939,7 @@
       <c r="O28" s="10"/>
       <c r="P28" s="6"/>
     </row>
-    <row r="29" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>50</v>
       </c>
@@ -2883,7 +2982,7 @@
       <c r="O29" s="8"/>
       <c r="P29" s="6"/>
     </row>
-    <row r="30" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>50</v>
       </c>
@@ -2925,7 +3024,7 @@
       </c>
       <c r="P30" s="6"/>
     </row>
-    <row r="31" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>50</v>
       </c>
@@ -2968,7 +3067,7 @@
       <c r="O31" s="10"/>
       <c r="P31" s="6"/>
     </row>
-    <row r="32" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>50</v>
       </c>
@@ -3011,7 +3110,7 @@
       <c r="O32" s="8"/>
       <c r="P32" s="6"/>
     </row>
-    <row r="33" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>50</v>
       </c>
@@ -3053,7 +3152,7 @@
       </c>
       <c r="P33" s="6"/>
     </row>
-    <row r="34" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>50</v>
       </c>
@@ -3096,7 +3195,7 @@
       <c r="O34" s="10"/>
       <c r="P34" s="6"/>
     </row>
-    <row r="35" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>50</v>
       </c>
@@ -3139,7 +3238,7 @@
       <c r="O35" s="8"/>
       <c r="P35" s="6"/>
     </row>
-    <row r="36" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>50</v>
       </c>
@@ -3181,7 +3280,7 @@
       </c>
       <c r="P36" s="6"/>
     </row>
-    <row r="37" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>50</v>
       </c>
@@ -3224,7 +3323,7 @@
       <c r="O37" s="10"/>
       <c r="P37" s="6"/>
     </row>
-    <row r="38" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>50</v>
       </c>
@@ -3267,7 +3366,7 @@
       <c r="O38" s="8"/>
       <c r="P38" s="6"/>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>69</v>
       </c>
@@ -3309,7 +3408,7 @@
       </c>
       <c r="P39" s="6"/>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>69</v>
       </c>
@@ -3352,7 +3451,7 @@
       <c r="O40" s="10"/>
       <c r="P40" s="6"/>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>69</v>
       </c>
@@ -3395,7 +3494,7 @@
       <c r="O41" s="8"/>
       <c r="P41" s="6"/>
     </row>
-    <row r="42" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>69</v>
       </c>
@@ -3437,7 +3536,7 @@
       </c>
       <c r="P42" s="6"/>
     </row>
-    <row r="43" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>69</v>
       </c>
@@ -3480,7 +3579,7 @@
       <c r="O43" s="10"/>
       <c r="P43" s="6"/>
     </row>
-    <row r="44" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>69</v>
       </c>
@@ -3523,7 +3622,7 @@
       <c r="O44" s="8"/>
       <c r="P44" s="6"/>
     </row>
-    <row r="45" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>69</v>
       </c>
@@ -3565,7 +3664,7 @@
       </c>
       <c r="P45" s="6"/>
     </row>
-    <row r="46" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>69</v>
       </c>
@@ -3608,7 +3707,7 @@
       <c r="O46" s="10"/>
       <c r="P46" s="6"/>
     </row>
-    <row r="47" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>69</v>
       </c>
@@ -3651,7 +3750,7 @@
       <c r="O47" s="8"/>
       <c r="P47" s="6"/>
     </row>
-    <row r="48" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>69</v>
       </c>
@@ -3693,7 +3792,7 @@
       </c>
       <c r="P48" s="6"/>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>81</v>
       </c>
@@ -3736,7 +3835,7 @@
       <c r="O49" s="10"/>
       <c r="P49" s="6"/>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>81</v>
       </c>
@@ -3779,7 +3878,7 @@
       <c r="O50" s="8"/>
       <c r="P50" s="6"/>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>81</v>
       </c>
@@ -3821,7 +3920,7 @@
       </c>
       <c r="P51" s="6"/>
     </row>
-    <row r="52" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>81</v>
       </c>
@@ -3864,7 +3963,7 @@
       <c r="O52" s="10"/>
       <c r="P52" s="6"/>
     </row>
-    <row r="53" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>81</v>
       </c>
@@ -3907,7 +4006,7 @@
       <c r="O53" s="8"/>
       <c r="P53" s="6"/>
     </row>
-    <row r="54" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>81</v>
       </c>
@@ -3949,7 +4048,7 @@
       </c>
       <c r="P54" s="6"/>
     </row>
-    <row r="55" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>81</v>
       </c>
@@ -3992,7 +4091,7 @@
       <c r="O55" s="10"/>
       <c r="P55" s="6"/>
     </row>
-    <row r="56" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>81</v>
       </c>
@@ -4035,7 +4134,7 @@
       <c r="O56" s="8"/>
       <c r="P56" s="6"/>
     </row>
-    <row r="57" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>81</v>
       </c>
@@ -4077,7 +4176,7 @@
       </c>
       <c r="P57" s="6"/>
     </row>
-    <row r="58" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>81</v>
       </c>
@@ -4120,7 +4219,7 @@
       <c r="O58" s="10"/>
       <c r="P58" s="6"/>
     </row>
-    <row r="59" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>81</v>
       </c>
@@ -4163,7 +4262,7 @@
       <c r="O59" s="8"/>
       <c r="P59" s="6"/>
     </row>
-    <row r="60" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>81</v>
       </c>
@@ -4205,7 +4304,7 @@
       </c>
       <c r="P60" s="6"/>
     </row>
-    <row r="61" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>81</v>
       </c>
@@ -4248,7 +4347,7 @@
       <c r="O61" s="10"/>
       <c r="P61" s="6"/>
     </row>
-    <row r="62" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>81</v>
       </c>
@@ -4291,7 +4390,7 @@
       <c r="O62" s="8"/>
       <c r="P62" s="6"/>
     </row>
-    <row r="63" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>81</v>
       </c>
@@ -4333,7 +4432,7 @@
       </c>
       <c r="P63" s="6"/>
     </row>
-    <row r="64" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>81</v>
       </c>
@@ -4376,7 +4475,7 @@
       <c r="O64" s="10"/>
       <c r="P64" s="6"/>
     </row>
-    <row r="65" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>81</v>
       </c>
@@ -4419,7 +4518,7 @@
       <c r="O65" s="8"/>
       <c r="P65" s="6"/>
     </row>
-    <row r="66" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>81</v>
       </c>
@@ -4461,7 +4560,7 @@
       </c>
       <c r="P66" s="6"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>100</v>
       </c>
@@ -4504,7 +4603,7 @@
       <c r="O67" s="10"/>
       <c r="P67" s="6"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>100</v>
       </c>
@@ -4547,7 +4646,7 @@
       <c r="O68" s="8"/>
       <c r="P68" s="6"/>
     </row>
-    <row r="69" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>100</v>
       </c>
@@ -4589,7 +4688,7 @@
       </c>
       <c r="P69" s="6"/>
     </row>
-    <row r="70" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>100</v>
       </c>
@@ -4632,7 +4731,7 @@
       <c r="O70" s="10"/>
       <c r="P70" s="6"/>
     </row>
-    <row r="71" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>100</v>
       </c>
@@ -4675,7 +4774,7 @@
       <c r="O71" s="8"/>
       <c r="P71" s="6"/>
     </row>
-    <row r="72" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>100</v>
       </c>
@@ -4717,7 +4816,7 @@
       </c>
       <c r="P72" s="6"/>
     </row>
-    <row r="73" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>100</v>
       </c>
@@ -4760,7 +4859,7 @@
       <c r="O73" s="10"/>
       <c r="P73" s="6"/>
     </row>
-    <row r="74" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>100</v>
       </c>
@@ -4803,7 +4902,7 @@
       <c r="O74" s="8"/>
       <c r="P74" s="6"/>
     </row>
-    <row r="75" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>100</v>
       </c>
@@ -4845,7 +4944,7 @@
       </c>
       <c r="P75" s="6"/>
     </row>
-    <row r="76" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>100</v>
       </c>
@@ -4888,7 +4987,7 @@
       <c r="O76" s="10"/>
       <c r="P76" s="6"/>
     </row>
-    <row r="77" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>100</v>
       </c>
@@ -4931,7 +5030,7 @@
       <c r="O77" s="8"/>
       <c r="P77" s="6"/>
     </row>
-    <row r="78" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>100</v>
       </c>
@@ -4973,7 +5072,7 @@
       </c>
       <c r="P78" s="6"/>
     </row>
-    <row r="79" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>100</v>
       </c>
@@ -5016,7 +5115,7 @@
       <c r="O79" s="10"/>
       <c r="P79" s="6"/>
     </row>
-    <row r="80" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>100</v>
       </c>
@@ -5059,7 +5158,7 @@
       <c r="O80" s="8"/>
       <c r="P80" s="6"/>
     </row>
-    <row r="81" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>100</v>
       </c>
@@ -5101,7 +5200,7 @@
       </c>
       <c r="P81" s="6"/>
     </row>
-    <row r="82" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>100</v>
       </c>
@@ -5144,7 +5243,7 @@
       <c r="O82" s="10"/>
       <c r="P82" s="6"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>81</v>
       </c>
@@ -5187,7 +5286,7 @@
       <c r="O83" s="8"/>
       <c r="P83" s="6"/>
     </row>
-    <row r="84" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>81</v>
       </c>
@@ -5229,7 +5328,7 @@
       </c>
       <c r="P84" s="6"/>
     </row>
-    <row r="85" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>119</v>
       </c>
@@ -5272,7 +5371,7 @@
       <c r="O85" s="10"/>
       <c r="P85" s="6"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>119</v>
       </c>
@@ -5280,7 +5379,7 @@
         <v>121</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D86" t="s">
         <v>289</v>
@@ -5315,7 +5414,7 @@
       <c r="O86" s="8"/>
       <c r="P86" s="6"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>119</v>
       </c>
@@ -5323,7 +5422,7 @@
         <v>122</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D87" t="s">
         <v>289</v>
@@ -5357,7 +5456,7 @@
       </c>
       <c r="P87" s="6"/>
     </row>
-    <row r="88" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>119</v>
       </c>
@@ -5365,7 +5464,7 @@
         <v>124</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>24</v>
+        <v>351</v>
       </c>
       <c r="D88" t="s">
         <v>289</v>
@@ -5400,7 +5499,7 @@
       <c r="O88" s="10"/>
       <c r="P88" s="6"/>
     </row>
-    <row r="89" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>119</v>
       </c>
@@ -5408,7 +5507,7 @@
         <v>125</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>24</v>
+        <v>351</v>
       </c>
       <c r="D89" t="s">
         <v>289</v>
@@ -5443,7 +5542,7 @@
       <c r="O89" s="8"/>
       <c r="P89" s="6"/>
     </row>
-    <row r="90" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>119</v>
       </c>
@@ -5485,7 +5584,7 @@
       </c>
       <c r="P90" s="6"/>
     </row>
-    <row r="91" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>119</v>
       </c>
@@ -5528,7 +5627,7 @@
       <c r="O91" s="10"/>
       <c r="P91" s="6"/>
     </row>
-    <row r="92" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>119</v>
       </c>
@@ -5571,7 +5670,7 @@
       <c r="O92" s="8"/>
       <c r="P92" s="6"/>
     </row>
-    <row r="93" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>119</v>
       </c>
@@ -5613,7 +5712,7 @@
       </c>
       <c r="P93" s="6"/>
     </row>
-    <row r="94" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>119</v>
       </c>
@@ -5656,7 +5755,7 @@
       <c r="O94" s="10"/>
       <c r="P94" s="6"/>
     </row>
-    <row r="95" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>119</v>
       </c>
@@ -5699,7 +5798,7 @@
       <c r="O95" s="8"/>
       <c r="P95" s="6"/>
     </row>
-    <row r="96" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>119</v>
       </c>
@@ -5741,7 +5840,7 @@
       </c>
       <c r="P96" s="6"/>
     </row>
-    <row r="97" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>119</v>
       </c>
@@ -5784,7 +5883,7 @@
       <c r="O97" s="10"/>
       <c r="P97" s="6"/>
     </row>
-    <row r="98" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>119</v>
       </c>
@@ -5827,7 +5926,7 @@
       <c r="O98" s="8"/>
       <c r="P98" s="6"/>
     </row>
-    <row r="99" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>119</v>
       </c>
@@ -5869,7 +5968,7 @@
       </c>
       <c r="P99" s="6"/>
     </row>
-    <row r="100" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>119</v>
       </c>
@@ -5912,7 +6011,7 @@
       <c r="O100" s="10"/>
       <c r="P100" s="6"/>
     </row>
-    <row r="101" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>119</v>
       </c>
@@ -5955,7 +6054,7 @@
       <c r="O101" s="8"/>
       <c r="P101" s="6"/>
     </row>
-    <row r="102" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>119</v>
       </c>
@@ -5997,7 +6096,7 @@
       </c>
       <c r="P102" s="6"/>
     </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>138</v>
       </c>
@@ -6005,7 +6104,7 @@
         <v>139</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D103" t="s">
         <v>291</v>
@@ -6040,7 +6139,7 @@
       <c r="O103" s="10"/>
       <c r="P103" s="6"/>
     </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>138</v>
       </c>
@@ -6048,7 +6147,7 @@
         <v>140</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D104" t="s">
         <v>291</v>
@@ -6083,7 +6182,7 @@
       <c r="O104" s="8"/>
       <c r="P104" s="6"/>
     </row>
-    <row r="105" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>138</v>
       </c>
@@ -6091,7 +6190,7 @@
         <v>141</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>24</v>
+        <v>352</v>
       </c>
       <c r="D105" t="s">
         <v>291</v>
@@ -6125,7 +6224,7 @@
       </c>
       <c r="P105" s="6"/>
     </row>
-    <row r="106" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>138</v>
       </c>
@@ -6133,7 +6232,7 @@
         <v>142</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>24</v>
+        <v>352</v>
       </c>
       <c r="D106" t="s">
         <v>291</v>
@@ -6168,7 +6267,7 @@
       <c r="O106" s="10"/>
       <c r="P106" s="6"/>
     </row>
-    <row r="107" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>138</v>
       </c>
@@ -6211,7 +6310,7 @@
       <c r="O107" s="8"/>
       <c r="P107" s="6"/>
     </row>
-    <row r="108" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>138</v>
       </c>
@@ -6253,7 +6352,7 @@
       </c>
       <c r="P108" s="6"/>
     </row>
-    <row r="109" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>138</v>
       </c>
@@ -6296,7 +6395,7 @@
       <c r="O109" s="10"/>
       <c r="P109" s="6"/>
     </row>
-    <row r="110" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>138</v>
       </c>
@@ -6339,7 +6438,7 @@
       <c r="O110" s="8"/>
       <c r="P110" s="6"/>
     </row>
-    <row r="111" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>138</v>
       </c>
@@ -6381,7 +6480,7 @@
       </c>
       <c r="P111" s="6"/>
     </row>
-    <row r="112" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>138</v>
       </c>
@@ -6424,7 +6523,7 @@
       <c r="O112" s="10"/>
       <c r="P112" s="6"/>
     </row>
-    <row r="113" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>138</v>
       </c>
@@ -6467,7 +6566,7 @@
       <c r="O113" s="8"/>
       <c r="P113" s="6"/>
     </row>
-    <row r="114" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>138</v>
       </c>
@@ -6509,7 +6608,7 @@
       </c>
       <c r="P114" s="6"/>
     </row>
-    <row r="115" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>138</v>
       </c>
@@ -6552,7 +6651,7 @@
       <c r="O115" s="10"/>
       <c r="P115" s="6"/>
     </row>
-    <row r="116" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>138</v>
       </c>
@@ -6595,7 +6694,7 @@
       <c r="O116" s="8"/>
       <c r="P116" s="6"/>
     </row>
-    <row r="117" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>138</v>
       </c>
@@ -6637,7 +6736,7 @@
       </c>
       <c r="P117" s="6"/>
     </row>
-    <row r="118" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>138</v>
       </c>
@@ -6680,7 +6779,7 @@
       <c r="O118" s="10"/>
       <c r="P118" s="6"/>
     </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>155</v>
       </c>
@@ -6688,7 +6787,7 @@
         <v>156</v>
       </c>
       <c r="C119" s="5" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D119" t="s">
         <v>290</v>
@@ -6723,7 +6822,7 @@
       <c r="O119" s="8"/>
       <c r="P119" s="6"/>
     </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>155</v>
       </c>
@@ -6731,7 +6830,7 @@
         <v>157</v>
       </c>
       <c r="C120" s="5" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D120" t="s">
         <v>290</v>
@@ -6765,7 +6864,7 @@
       </c>
       <c r="P120" s="6"/>
     </row>
-    <row r="121" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>155</v>
       </c>
@@ -6773,7 +6872,7 @@
         <v>158</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>24</v>
+        <v>352</v>
       </c>
       <c r="D121" t="s">
         <v>290</v>
@@ -6808,7 +6907,7 @@
       <c r="O121" s="10"/>
       <c r="P121" s="6"/>
     </row>
-    <row r="122" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>155</v>
       </c>
@@ -6816,7 +6915,7 @@
         <v>159</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>24</v>
+        <v>352</v>
       </c>
       <c r="D122" t="s">
         <v>290</v>
@@ -6851,7 +6950,7 @@
       <c r="O122" s="8"/>
       <c r="P122" s="6"/>
     </row>
-    <row r="123" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>155</v>
       </c>
@@ -6893,7 +6992,7 @@
       </c>
       <c r="P123" s="6"/>
     </row>
-    <row r="124" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>155</v>
       </c>
@@ -6936,7 +7035,7 @@
       <c r="O124" s="10"/>
       <c r="P124" s="6"/>
     </row>
-    <row r="125" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>155</v>
       </c>
@@ -6979,7 +7078,7 @@
       <c r="O125" s="8"/>
       <c r="P125" s="6"/>
     </row>
-    <row r="126" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>155</v>
       </c>
@@ -7021,7 +7120,7 @@
       </c>
       <c r="P126" s="6"/>
     </row>
-    <row r="127" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>155</v>
       </c>
@@ -7064,7 +7163,7 @@
       <c r="O127" s="10"/>
       <c r="P127" s="6"/>
     </row>
-    <row r="128" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>155</v>
       </c>
@@ -7107,7 +7206,7 @@
       <c r="O128" s="8"/>
       <c r="P128" s="6"/>
     </row>
-    <row r="129" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>155</v>
       </c>
@@ -7149,7 +7248,7 @@
       </c>
       <c r="P129" s="6"/>
     </row>
-    <row r="130" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>155</v>
       </c>
@@ -7192,7 +7291,7 @@
       <c r="O130" s="10"/>
       <c r="P130" s="6"/>
     </row>
-    <row r="131" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>155</v>
       </c>
@@ -7235,7 +7334,7 @@
       <c r="O131" s="8"/>
       <c r="P131" s="6"/>
     </row>
-    <row r="132" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>155</v>
       </c>
@@ -7277,7 +7376,7 @@
       </c>
       <c r="P132" s="6"/>
     </row>
-    <row r="133" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>155</v>
       </c>
@@ -7320,7 +7419,7 @@
       <c r="O133" s="10"/>
       <c r="P133" s="6"/>
     </row>
-    <row r="134" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>155</v>
       </c>
@@ -7363,7 +7462,7 @@
       <c r="O134" s="8"/>
       <c r="P134" s="6"/>
     </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>138</v>
       </c>
@@ -7405,7 +7504,7 @@
       </c>
       <c r="P135" s="6"/>
     </row>
-    <row r="136" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>138</v>
       </c>
@@ -7448,7 +7547,7 @@
       <c r="O136" s="10"/>
       <c r="P136" s="6"/>
     </row>
-    <row r="137" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>172</v>
       </c>
@@ -7491,7 +7590,7 @@
       <c r="O137" s="8"/>
       <c r="P137" s="6"/>
     </row>
-    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>172</v>
       </c>
@@ -7533,7 +7632,7 @@
       </c>
       <c r="P138" s="6"/>
     </row>
-    <row r="139" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>172</v>
       </c>
@@ -7576,7 +7675,7 @@
       <c r="O139" s="10"/>
       <c r="P139" s="6"/>
     </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>172</v>
       </c>
@@ -7619,7 +7718,7 @@
       <c r="O140" s="8"/>
       <c r="P140" s="6"/>
     </row>
-    <row r="141" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>172</v>
       </c>
@@ -7661,7 +7760,7 @@
       </c>
       <c r="P141" s="6"/>
     </row>
-    <row r="142" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>172</v>
       </c>
@@ -7704,7 +7803,7 @@
       <c r="O142" s="10"/>
       <c r="P142" s="6"/>
     </row>
-    <row r="143" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>172</v>
       </c>
@@ -7747,7 +7846,7 @@
       <c r="O143" s="8"/>
       <c r="P143" s="6"/>
     </row>
-    <row r="144" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>172</v>
       </c>
@@ -7789,7 +7888,7 @@
       </c>
       <c r="P144" s="6"/>
     </row>
-    <row r="145" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>172</v>
       </c>
@@ -7832,7 +7931,7 @@
       <c r="O145" s="10"/>
       <c r="P145" s="6"/>
     </row>
-    <row r="146" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>172</v>
       </c>
@@ -7875,7 +7974,7 @@
       <c r="O146" s="8"/>
       <c r="P146" s="6"/>
     </row>
-    <row r="147" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>172</v>
       </c>
@@ -7917,7 +8016,7 @@
       </c>
       <c r="P147" s="6"/>
     </row>
-    <row r="148" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>172</v>
       </c>
@@ -7960,7 +8059,7 @@
       <c r="O148" s="10"/>
       <c r="P148" s="6"/>
     </row>
-    <row r="149" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>172</v>
       </c>
@@ -8003,7 +8102,7 @@
       <c r="O149" s="8"/>
       <c r="P149" s="6"/>
     </row>
-    <row r="150" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>172</v>
       </c>
@@ -8045,7 +8144,7 @@
       </c>
       <c r="P150" s="6"/>
     </row>
-    <row r="151" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>172</v>
       </c>
@@ -8088,7 +8187,7 @@
       <c r="O151" s="10"/>
       <c r="P151" s="6"/>
     </row>
-    <row r="152" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>172</v>
       </c>
@@ -8131,7 +8230,7 @@
       <c r="O152" s="8"/>
       <c r="P152" s="6"/>
     </row>
-    <row r="153" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>176</v>
       </c>
@@ -8173,7 +8272,7 @@
       </c>
       <c r="P153" s="6"/>
     </row>
-    <row r="154" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>176</v>
       </c>
@@ -8216,7 +8315,7 @@
       <c r="O154" s="10"/>
       <c r="P154" s="6"/>
     </row>
-    <row r="155" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>176</v>
       </c>
@@ -8259,7 +8358,7 @@
       <c r="O155" s="8"/>
       <c r="P155" s="6"/>
     </row>
-    <row r="156" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>176</v>
       </c>
@@ -8301,7 +8400,7 @@
       </c>
       <c r="P156" s="6"/>
     </row>
-    <row r="157" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>176</v>
       </c>
@@ -8344,7 +8443,7 @@
       <c r="O157" s="10"/>
       <c r="P157" s="6"/>
     </row>
-    <row r="158" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>176</v>
       </c>
@@ -8387,7 +8486,7 @@
       <c r="O158" s="8"/>
       <c r="P158" s="6"/>
     </row>
-    <row r="159" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>176</v>
       </c>
@@ -8429,7 +8528,7 @@
       </c>
       <c r="P159" s="6"/>
     </row>
-    <row r="160" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>176</v>
       </c>
@@ -8472,7 +8571,7 @@
       <c r="O160" s="10"/>
       <c r="P160" s="6"/>
     </row>
-    <row r="161" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>176</v>
       </c>
@@ -8515,7 +8614,7 @@
       <c r="O161" s="8"/>
       <c r="P161" s="6"/>
     </row>
-    <row r="162" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>176</v>
       </c>
@@ -8557,7 +8656,7 @@
       </c>
       <c r="P162" s="6"/>
     </row>
-    <row r="163" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>176</v>
       </c>
@@ -8600,7 +8699,7 @@
       <c r="O163" s="10"/>
       <c r="P163" s="6"/>
     </row>
-    <row r="164" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>176</v>
       </c>
@@ -8643,7 +8742,7 @@
       <c r="O164" s="8"/>
       <c r="P164" s="6"/>
     </row>
-    <row r="165" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>176</v>
       </c>
@@ -8685,7 +8784,7 @@
       </c>
       <c r="P165" s="6"/>
     </row>
-    <row r="166" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>176</v>
       </c>
@@ -8728,7 +8827,7 @@
       <c r="O166" s="10"/>
       <c r="P166" s="6"/>
     </row>
-    <row r="167" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>176</v>
       </c>
@@ -8771,7 +8870,7 @@
       <c r="O167" s="8"/>
       <c r="P167" s="6"/>
     </row>
-    <row r="168" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>176</v>
       </c>
@@ -8813,7 +8912,7 @@
       </c>
       <c r="P168" s="6"/>
     </row>
-    <row r="169" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>178</v>
       </c>
@@ -8856,7 +8955,7 @@
       <c r="O169" s="10"/>
       <c r="P169" s="6"/>
     </row>
-    <row r="170" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>178</v>
       </c>
@@ -8899,7 +8998,7 @@
       <c r="O170" s="8"/>
       <c r="P170" s="6"/>
     </row>
-    <row r="171" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>178</v>
       </c>
@@ -8941,7 +9040,7 @@
       </c>
       <c r="P171" s="6"/>
     </row>
-    <row r="172" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>178</v>
       </c>
@@ -8984,7 +9083,7 @@
       <c r="O172" s="10"/>
       <c r="P172" s="6"/>
     </row>
-    <row r="173" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>178</v>
       </c>
@@ -9027,7 +9126,7 @@
       <c r="O173" s="8"/>
       <c r="P173" s="6"/>
     </row>
-    <row r="174" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>178</v>
       </c>
@@ -9069,7 +9168,7 @@
       </c>
       <c r="P174" s="6"/>
     </row>
-    <row r="175" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>178</v>
       </c>
@@ -9112,7 +9211,7 @@
       <c r="O175" s="10"/>
       <c r="P175" s="6"/>
     </row>
-    <row r="176" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>178</v>
       </c>
@@ -9155,7 +9254,7 @@
       <c r="O176" s="8"/>
       <c r="P176" s="6"/>
     </row>
-    <row r="177" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>178</v>
       </c>
@@ -9197,7 +9296,7 @@
       </c>
       <c r="P177" s="6"/>
     </row>
-    <row r="178" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>178</v>
       </c>
@@ -9240,7 +9339,7 @@
       <c r="O178" s="10"/>
       <c r="P178" s="6"/>
     </row>
-    <row r="179" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>178</v>
       </c>
@@ -9283,7 +9382,7 @@
       <c r="O179" s="8"/>
       <c r="P179" s="6"/>
     </row>
-    <row r="180" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>178</v>
       </c>
@@ -9325,7 +9424,7 @@
       </c>
       <c r="P180" s="6"/>
     </row>
-    <row r="181" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>178</v>
       </c>
@@ -9368,7 +9467,7 @@
       <c r="O181" s="10"/>
       <c r="P181" s="6"/>
     </row>
-    <row r="182" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>178</v>
       </c>
@@ -9411,7 +9510,7 @@
       <c r="O182" s="8"/>
       <c r="P182" s="6"/>
     </row>
-    <row r="183" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>178</v>
       </c>
@@ -9453,7 +9552,7 @@
       </c>
       <c r="P183" s="6"/>
     </row>
-    <row r="184" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>178</v>
       </c>
@@ -9496,7 +9595,7 @@
       <c r="O184" s="10"/>
       <c r="P184" s="6"/>
     </row>
-    <row r="185" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>179</v>
       </c>
@@ -9539,7 +9638,7 @@
       <c r="O185" s="8"/>
       <c r="P185" s="6"/>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>179</v>
       </c>
@@ -9581,7 +9680,7 @@
       </c>
       <c r="P186" s="6"/>
     </row>
-    <row r="187" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>179</v>
       </c>
@@ -9624,7 +9723,7 @@
       <c r="O187" s="10"/>
       <c r="P187" s="6"/>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>179</v>
       </c>
@@ -9667,7 +9766,7 @@
       <c r="O188" s="8"/>
       <c r="P188" s="6"/>
     </row>
-    <row r="189" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>179</v>
       </c>
@@ -9709,7 +9808,7 @@
       </c>
       <c r="P189" s="6"/>
     </row>
-    <row r="190" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>179</v>
       </c>
@@ -9752,7 +9851,7 @@
       <c r="O190" s="10"/>
       <c r="P190" s="6"/>
     </row>
-    <row r="191" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>179</v>
       </c>
@@ -9795,7 +9894,7 @@
       <c r="O191" s="8"/>
       <c r="P191" s="6"/>
     </row>
-    <row r="192" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>179</v>
       </c>
@@ -9837,7 +9936,7 @@
       </c>
       <c r="P192" s="6"/>
     </row>
-    <row r="193" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>179</v>
       </c>
@@ -9880,7 +9979,7 @@
       <c r="O193" s="10"/>
       <c r="P193" s="6"/>
     </row>
-    <row r="194" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>179</v>
       </c>
@@ -9923,7 +10022,7 @@
       <c r="O194" s="8"/>
       <c r="P194" s="6"/>
     </row>
-    <row r="195" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>179</v>
       </c>
@@ -9965,7 +10064,7 @@
       </c>
       <c r="P195" s="6"/>
     </row>
-    <row r="196" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>179</v>
       </c>
@@ -10008,7 +10107,7 @@
       <c r="O196" s="10"/>
       <c r="P196" s="6"/>
     </row>
-    <row r="197" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>179</v>
       </c>
@@ -10051,7 +10150,7 @@
       <c r="O197" s="8"/>
       <c r="P197" s="6"/>
     </row>
-    <row r="198" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>179</v>
       </c>
@@ -10093,7 +10192,7 @@
       </c>
       <c r="P198" s="6"/>
     </row>
-    <row r="199" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>179</v>
       </c>
@@ -10136,7 +10235,7 @@
       <c r="O199" s="10"/>
       <c r="P199" s="6"/>
     </row>
-    <row r="200" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>179</v>
       </c>
@@ -10179,7 +10278,7 @@
       <c r="O200" s="8"/>
       <c r="P200" s="6"/>
     </row>
-    <row r="201" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>172</v>
       </c>
@@ -10221,7 +10320,7 @@
       </c>
       <c r="P201" s="6"/>
     </row>
-    <row r="202" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>172</v>
       </c>
@@ -10264,7 +10363,7 @@
       <c r="O202" s="10"/>
       <c r="P202" s="6"/>
     </row>
-    <row r="203" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>179</v>
       </c>
@@ -10307,7 +10406,7 @@
       <c r="O203" s="8"/>
       <c r="P203" s="6"/>
     </row>
-    <row r="204" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>179</v>
       </c>
@@ -10349,7 +10448,7 @@
       </c>
       <c r="P204" s="6"/>
     </row>
-    <row r="205" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>260</v>
       </c>
@@ -10392,7 +10491,7 @@
       <c r="O205" s="10"/>
       <c r="P205" s="6"/>
     </row>
-    <row r="206" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>260</v>
       </c>
@@ -10435,7 +10534,7 @@
       <c r="O206" s="8"/>
       <c r="P206" s="6"/>
     </row>
-    <row r="207" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>260</v>
       </c>
@@ -10477,7 +10576,7 @@
       </c>
       <c r="P207" s="6"/>
     </row>
-    <row r="208" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>260</v>
       </c>
@@ -10520,7 +10619,7 @@
       <c r="O208" s="10"/>
       <c r="P208" s="6"/>
     </row>
-    <row r="209" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>260</v>
       </c>
@@ -10563,7 +10662,7 @@
       <c r="O209" s="8"/>
       <c r="P209" s="6"/>
     </row>
-    <row r="210" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>260</v>
       </c>
@@ -10605,7 +10704,7 @@
       </c>
       <c r="P210" s="6"/>
     </row>
-    <row r="211" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>260</v>
       </c>
@@ -10648,7 +10747,7 @@
       <c r="O211" s="10"/>
       <c r="P211" s="6"/>
     </row>
-    <row r="212" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>260</v>
       </c>
@@ -10691,7 +10790,7 @@
       <c r="O212" s="8"/>
       <c r="P212" s="6"/>
     </row>
-    <row r="213" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>277</v>
       </c>
@@ -10733,7 +10832,7 @@
       </c>
       <c r="P213" s="6"/>
     </row>
-    <row r="214" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>277</v>
       </c>
@@ -10776,7 +10875,7 @@
       <c r="O214" s="10"/>
       <c r="P214" s="6"/>
     </row>
-    <row r="215" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>277</v>
       </c>
@@ -10819,7 +10918,7 @@
       <c r="O215" s="8"/>
       <c r="P215" s="6"/>
     </row>
-    <row r="216" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>277</v>
       </c>
@@ -10861,7 +10960,7 @@
       </c>
       <c r="P216" s="6"/>
     </row>
-    <row r="217" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>277</v>
       </c>
@@ -10904,7 +11003,7 @@
       <c r="O217" s="10"/>
       <c r="P217" s="6"/>
     </row>
-    <row r="218" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>277</v>
       </c>
@@ -10947,7 +11046,7 @@
       <c r="O218" s="8"/>
       <c r="P218" s="6"/>
     </row>
-    <row r="219" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>277</v>
       </c>
@@ -10989,7 +11088,7 @@
       </c>
       <c r="P219" s="6"/>
     </row>
-    <row r="220" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>277</v>
       </c>
@@ -11032,7 +11131,7 @@
       <c r="O220" s="10"/>
       <c r="P220" s="6"/>
     </row>
-    <row r="221" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>303</v>
       </c>
@@ -11075,7 +11174,7 @@
       <c r="O221" s="8"/>
       <c r="P221" s="6"/>
     </row>
-    <row r="222" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>303</v>
       </c>
@@ -11117,7 +11216,7 @@
       </c>
       <c r="P222" s="6"/>
     </row>
-    <row r="223" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
         <v>303</v>
       </c>
@@ -11160,7 +11259,7 @@
       <c r="O223" s="10"/>
       <c r="P223" s="6"/>
     </row>
-    <row r="224" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>303</v>
       </c>
@@ -11203,7 +11302,7 @@
       <c r="O224" s="8"/>
       <c r="P224" s="6"/>
     </row>
-    <row r="225" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>303</v>
       </c>
@@ -11245,7 +11344,7 @@
       </c>
       <c r="P225" s="6"/>
     </row>
-    <row r="226" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>303</v>
       </c>
@@ -11288,7 +11387,7 @@
       <c r="O226" s="10"/>
       <c r="P226" s="6"/>
     </row>
-    <row r="227" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>303</v>
       </c>
@@ -11331,7 +11430,7 @@
       <c r="O227" s="8"/>
       <c r="P227" s="6"/>
     </row>
-    <row r="228" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>303</v>
       </c>
@@ -11373,7 +11472,7 @@
       </c>
       <c r="P228" s="6"/>
     </row>
-    <row r="229" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>303</v>
       </c>
@@ -11416,7 +11515,7 @@
       <c r="O229" s="10"/>
       <c r="P229" s="6"/>
     </row>
-    <row r="230" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>303</v>
       </c>
@@ -11459,7 +11558,7 @@
       <c r="O230" s="8"/>
       <c r="P230" s="6"/>
     </row>
-    <row r="231" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>303</v>
       </c>
@@ -11501,7 +11600,7 @@
       </c>
       <c r="P231" s="6"/>
     </row>
-    <row r="232" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>303</v>
       </c>
@@ -11544,7 +11643,7 @@
       <c r="O232" s="10"/>
       <c r="P232" s="6"/>
     </row>
-    <row r="233" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>303</v>
       </c>
@@ -11587,7 +11686,7 @@
       <c r="O233" s="8"/>
       <c r="P233" s="6"/>
     </row>
-    <row r="234" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>303</v>
       </c>
@@ -11629,7 +11728,7 @@
       </c>
       <c r="P234" s="6"/>
     </row>
-    <row r="235" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>303</v>
       </c>
@@ -11672,7 +11771,7 @@
       <c r="O235" s="10"/>
       <c r="P235" s="6"/>
     </row>
-    <row r="236" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>303</v>
       </c>
@@ -11715,8 +11814,1156 @@
       <c r="O236" s="8"/>
       <c r="P236" s="6"/>
     </row>
+    <row r="237" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A237" t="s">
+        <v>69</v>
+      </c>
+      <c r="B237" t="s">
+        <v>321</v>
+      </c>
+      <c r="C237" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D237" t="s">
+        <v>289</v>
+      </c>
+      <c r="E237" t="s">
+        <v>16</v>
+      </c>
+      <c r="F237" t="s">
+        <v>71</v>
+      </c>
+      <c r="G237" t="s">
+        <v>300</v>
+      </c>
+      <c r="H237" t="s">
+        <v>18</v>
+      </c>
+      <c r="I237" t="s">
+        <v>19</v>
+      </c>
+      <c r="J237" t="s">
+        <v>322</v>
+      </c>
+      <c r="K237" t="s">
+        <v>20</v>
+      </c>
+      <c r="L237" t="s">
+        <v>21</v>
+      </c>
+      <c r="M237" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="238" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A238" t="s">
+        <v>69</v>
+      </c>
+      <c r="B238" t="s">
+        <v>323</v>
+      </c>
+      <c r="C238" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D238" t="s">
+        <v>289</v>
+      </c>
+      <c r="E238" t="s">
+        <v>16</v>
+      </c>
+      <c r="F238" t="s">
+        <v>71</v>
+      </c>
+      <c r="G238" t="s">
+        <v>300</v>
+      </c>
+      <c r="H238" t="s">
+        <v>18</v>
+      </c>
+      <c r="I238" t="s">
+        <v>19</v>
+      </c>
+      <c r="J238" t="s">
+        <v>322</v>
+      </c>
+      <c r="K238" t="s">
+        <v>30</v>
+      </c>
+      <c r="L238" t="s">
+        <v>21</v>
+      </c>
+      <c r="M238" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="239" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A239" t="s">
+        <v>69</v>
+      </c>
+      <c r="B239" t="s">
+        <v>324</v>
+      </c>
+      <c r="C239" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D239" t="s">
+        <v>289</v>
+      </c>
+      <c r="E239" t="s">
+        <v>16</v>
+      </c>
+      <c r="F239" t="s">
+        <v>71</v>
+      </c>
+      <c r="G239" t="s">
+        <v>300</v>
+      </c>
+      <c r="H239" t="s">
+        <v>18</v>
+      </c>
+      <c r="I239" t="s">
+        <v>19</v>
+      </c>
+      <c r="J239" t="s">
+        <v>322</v>
+      </c>
+      <c r="K239" t="s">
+        <v>30</v>
+      </c>
+      <c r="L239" t="s">
+        <v>21</v>
+      </c>
+      <c r="M239" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="240" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A240" t="s">
+        <v>69</v>
+      </c>
+      <c r="B240" t="s">
+        <v>325</v>
+      </c>
+      <c r="C240" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D240" t="s">
+        <v>289</v>
+      </c>
+      <c r="E240" t="s">
+        <v>16</v>
+      </c>
+      <c r="F240" t="s">
+        <v>71</v>
+      </c>
+      <c r="G240" t="s">
+        <v>300</v>
+      </c>
+      <c r="H240" t="s">
+        <v>18</v>
+      </c>
+      <c r="I240" t="s">
+        <v>19</v>
+      </c>
+      <c r="J240" t="s">
+        <v>322</v>
+      </c>
+      <c r="K240" t="s">
+        <v>20</v>
+      </c>
+      <c r="L240" t="s">
+        <v>21</v>
+      </c>
+      <c r="M240" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="241" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A241" t="s">
+        <v>119</v>
+      </c>
+      <c r="B241" t="s">
+        <v>326</v>
+      </c>
+      <c r="C241" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D241" t="s">
+        <v>289</v>
+      </c>
+      <c r="E241" t="s">
+        <v>52</v>
+      </c>
+      <c r="F241" t="s">
+        <v>120</v>
+      </c>
+      <c r="G241" t="s">
+        <v>17</v>
+      </c>
+      <c r="H241" t="s">
+        <v>18</v>
+      </c>
+      <c r="I241" t="s">
+        <v>53</v>
+      </c>
+      <c r="J241" t="s">
+        <v>322</v>
+      </c>
+      <c r="K241" t="s">
+        <v>20</v>
+      </c>
+      <c r="L241" t="s">
+        <v>21</v>
+      </c>
+      <c r="M241" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="242" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A242" t="s">
+        <v>119</v>
+      </c>
+      <c r="B242" t="s">
+        <v>327</v>
+      </c>
+      <c r="C242" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D242" t="s">
+        <v>289</v>
+      </c>
+      <c r="E242" t="s">
+        <v>52</v>
+      </c>
+      <c r="F242" t="s">
+        <v>120</v>
+      </c>
+      <c r="G242" t="s">
+        <v>17</v>
+      </c>
+      <c r="H242" t="s">
+        <v>18</v>
+      </c>
+      <c r="I242" t="s">
+        <v>53</v>
+      </c>
+      <c r="J242" t="s">
+        <v>322</v>
+      </c>
+      <c r="K242" t="s">
+        <v>30</v>
+      </c>
+      <c r="L242" t="s">
+        <v>21</v>
+      </c>
+      <c r="M242" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="243" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A243" t="s">
+        <v>119</v>
+      </c>
+      <c r="B243" t="s">
+        <v>328</v>
+      </c>
+      <c r="C243" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D243" t="s">
+        <v>289</v>
+      </c>
+      <c r="E243" t="s">
+        <v>52</v>
+      </c>
+      <c r="F243" t="s">
+        <v>120</v>
+      </c>
+      <c r="G243" t="s">
+        <v>17</v>
+      </c>
+      <c r="H243" t="s">
+        <v>18</v>
+      </c>
+      <c r="I243" t="s">
+        <v>19</v>
+      </c>
+      <c r="J243" t="s">
+        <v>322</v>
+      </c>
+      <c r="K243" t="s">
+        <v>30</v>
+      </c>
+      <c r="L243" t="s">
+        <v>21</v>
+      </c>
+      <c r="M243" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="244" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A244" t="s">
+        <v>119</v>
+      </c>
+      <c r="B244" t="s">
+        <v>329</v>
+      </c>
+      <c r="C244" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D244" t="s">
+        <v>289</v>
+      </c>
+      <c r="E244" t="s">
+        <v>52</v>
+      </c>
+      <c r="F244" t="s">
+        <v>120</v>
+      </c>
+      <c r="G244" t="s">
+        <v>17</v>
+      </c>
+      <c r="H244" t="s">
+        <v>18</v>
+      </c>
+      <c r="I244" t="s">
+        <v>19</v>
+      </c>
+      <c r="J244" t="s">
+        <v>322</v>
+      </c>
+      <c r="K244" t="s">
+        <v>20</v>
+      </c>
+      <c r="L244" t="s">
+        <v>21</v>
+      </c>
+      <c r="M244" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="245" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A245" t="s">
+        <v>119</v>
+      </c>
+      <c r="B245" t="s">
+        <v>330</v>
+      </c>
+      <c r="C245" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D245" t="s">
+        <v>289</v>
+      </c>
+      <c r="E245" t="s">
+        <v>52</v>
+      </c>
+      <c r="F245" t="s">
+        <v>120</v>
+      </c>
+      <c r="G245" t="s">
+        <v>17</v>
+      </c>
+      <c r="H245" t="s">
+        <v>18</v>
+      </c>
+      <c r="I245" t="s">
+        <v>53</v>
+      </c>
+      <c r="J245" t="s">
+        <v>322</v>
+      </c>
+      <c r="K245" t="s">
+        <v>30</v>
+      </c>
+      <c r="L245" t="s">
+        <v>21</v>
+      </c>
+      <c r="M245" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="246" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A246" t="s">
+        <v>119</v>
+      </c>
+      <c r="B246" t="s">
+        <v>331</v>
+      </c>
+      <c r="C246" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D246" t="s">
+        <v>289</v>
+      </c>
+      <c r="E246" t="s">
+        <v>52</v>
+      </c>
+      <c r="F246" t="s">
+        <v>120</v>
+      </c>
+      <c r="G246" t="s">
+        <v>17</v>
+      </c>
+      <c r="H246" t="s">
+        <v>18</v>
+      </c>
+      <c r="I246" t="s">
+        <v>53</v>
+      </c>
+      <c r="J246" t="s">
+        <v>322</v>
+      </c>
+      <c r="K246" t="s">
+        <v>20</v>
+      </c>
+      <c r="L246" t="s">
+        <v>21</v>
+      </c>
+      <c r="M246" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="247" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A247" t="s">
+        <v>119</v>
+      </c>
+      <c r="B247" t="s">
+        <v>332</v>
+      </c>
+      <c r="C247" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D247" t="s">
+        <v>289</v>
+      </c>
+      <c r="E247" t="s">
+        <v>52</v>
+      </c>
+      <c r="F247" t="s">
+        <v>120</v>
+      </c>
+      <c r="G247" t="s">
+        <v>17</v>
+      </c>
+      <c r="H247" t="s">
+        <v>18</v>
+      </c>
+      <c r="I247" t="s">
+        <v>19</v>
+      </c>
+      <c r="J247" t="s">
+        <v>322</v>
+      </c>
+      <c r="K247" t="s">
+        <v>30</v>
+      </c>
+      <c r="L247" t="s">
+        <v>21</v>
+      </c>
+      <c r="M247" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="248" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A248" t="s">
+        <v>119</v>
+      </c>
+      <c r="B248" t="s">
+        <v>333</v>
+      </c>
+      <c r="C248" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D248" t="s">
+        <v>289</v>
+      </c>
+      <c r="E248" t="s">
+        <v>52</v>
+      </c>
+      <c r="F248" t="s">
+        <v>120</v>
+      </c>
+      <c r="G248" t="s">
+        <v>17</v>
+      </c>
+      <c r="H248" t="s">
+        <v>18</v>
+      </c>
+      <c r="I248" t="s">
+        <v>19</v>
+      </c>
+      <c r="J248" t="s">
+        <v>322</v>
+      </c>
+      <c r="K248" t="s">
+        <v>20</v>
+      </c>
+      <c r="L248" t="s">
+        <v>21</v>
+      </c>
+      <c r="M248" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="249" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A249" t="s">
+        <v>138</v>
+      </c>
+      <c r="B249" t="s">
+        <v>334</v>
+      </c>
+      <c r="C249" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D249" t="s">
+        <v>291</v>
+      </c>
+      <c r="E249" t="s">
+        <v>52</v>
+      </c>
+      <c r="F249" t="s">
+        <v>120</v>
+      </c>
+      <c r="G249" t="s">
+        <v>17</v>
+      </c>
+      <c r="H249" t="s">
+        <v>18</v>
+      </c>
+      <c r="I249" t="s">
+        <v>53</v>
+      </c>
+      <c r="J249" t="s">
+        <v>322</v>
+      </c>
+      <c r="K249" t="s">
+        <v>20</v>
+      </c>
+      <c r="L249" t="s">
+        <v>21</v>
+      </c>
+      <c r="M249" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="250" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A250" t="s">
+        <v>138</v>
+      </c>
+      <c r="B250" t="s">
+        <v>335</v>
+      </c>
+      <c r="C250" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D250" t="s">
+        <v>291</v>
+      </c>
+      <c r="E250" t="s">
+        <v>52</v>
+      </c>
+      <c r="F250" t="s">
+        <v>120</v>
+      </c>
+      <c r="G250" t="s">
+        <v>17</v>
+      </c>
+      <c r="H250" t="s">
+        <v>18</v>
+      </c>
+      <c r="I250" t="s">
+        <v>53</v>
+      </c>
+      <c r="J250" t="s">
+        <v>322</v>
+      </c>
+      <c r="K250" t="s">
+        <v>30</v>
+      </c>
+      <c r="L250" t="s">
+        <v>21</v>
+      </c>
+      <c r="M250" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="251" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A251" t="s">
+        <v>138</v>
+      </c>
+      <c r="B251" t="s">
+        <v>336</v>
+      </c>
+      <c r="C251" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D251" t="s">
+        <v>291</v>
+      </c>
+      <c r="E251" t="s">
+        <v>52</v>
+      </c>
+      <c r="F251" t="s">
+        <v>120</v>
+      </c>
+      <c r="G251" t="s">
+        <v>17</v>
+      </c>
+      <c r="H251" t="s">
+        <v>18</v>
+      </c>
+      <c r="I251" t="s">
+        <v>19</v>
+      </c>
+      <c r="J251" t="s">
+        <v>322</v>
+      </c>
+      <c r="K251" t="s">
+        <v>30</v>
+      </c>
+      <c r="L251" t="s">
+        <v>21</v>
+      </c>
+      <c r="M251" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="252" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A252" t="s">
+        <v>138</v>
+      </c>
+      <c r="B252" t="s">
+        <v>337</v>
+      </c>
+      <c r="C252" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D252" t="s">
+        <v>291</v>
+      </c>
+      <c r="E252" t="s">
+        <v>52</v>
+      </c>
+      <c r="F252" t="s">
+        <v>120</v>
+      </c>
+      <c r="G252" t="s">
+        <v>17</v>
+      </c>
+      <c r="H252" t="s">
+        <v>18</v>
+      </c>
+      <c r="I252" t="s">
+        <v>19</v>
+      </c>
+      <c r="J252" t="s">
+        <v>322</v>
+      </c>
+      <c r="K252" t="s">
+        <v>20</v>
+      </c>
+      <c r="L252" t="s">
+        <v>21</v>
+      </c>
+      <c r="M252" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="253" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A253" t="s">
+        <v>138</v>
+      </c>
+      <c r="B253" t="s">
+        <v>338</v>
+      </c>
+      <c r="C253" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D253" t="s">
+        <v>291</v>
+      </c>
+      <c r="E253" t="s">
+        <v>52</v>
+      </c>
+      <c r="F253" t="s">
+        <v>120</v>
+      </c>
+      <c r="G253" t="s">
+        <v>17</v>
+      </c>
+      <c r="H253" t="s">
+        <v>18</v>
+      </c>
+      <c r="I253" t="s">
+        <v>53</v>
+      </c>
+      <c r="J253" t="s">
+        <v>322</v>
+      </c>
+      <c r="K253" t="s">
+        <v>30</v>
+      </c>
+      <c r="L253" t="s">
+        <v>21</v>
+      </c>
+      <c r="M253" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="254" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A254" t="s">
+        <v>138</v>
+      </c>
+      <c r="B254" t="s">
+        <v>339</v>
+      </c>
+      <c r="C254" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D254" t="s">
+        <v>291</v>
+      </c>
+      <c r="E254" t="s">
+        <v>52</v>
+      </c>
+      <c r="F254" t="s">
+        <v>120</v>
+      </c>
+      <c r="G254" t="s">
+        <v>17</v>
+      </c>
+      <c r="H254" t="s">
+        <v>18</v>
+      </c>
+      <c r="I254" t="s">
+        <v>53</v>
+      </c>
+      <c r="J254" t="s">
+        <v>322</v>
+      </c>
+      <c r="K254" t="s">
+        <v>20</v>
+      </c>
+      <c r="L254" t="s">
+        <v>21</v>
+      </c>
+      <c r="M254" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="255" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A255" t="s">
+        <v>138</v>
+      </c>
+      <c r="B255" t="s">
+        <v>340</v>
+      </c>
+      <c r="C255" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D255" t="s">
+        <v>291</v>
+      </c>
+      <c r="E255" t="s">
+        <v>52</v>
+      </c>
+      <c r="F255" t="s">
+        <v>120</v>
+      </c>
+      <c r="G255" t="s">
+        <v>17</v>
+      </c>
+      <c r="H255" t="s">
+        <v>18</v>
+      </c>
+      <c r="I255" t="s">
+        <v>19</v>
+      </c>
+      <c r="J255" t="s">
+        <v>322</v>
+      </c>
+      <c r="K255" t="s">
+        <v>30</v>
+      </c>
+      <c r="L255" t="s">
+        <v>21</v>
+      </c>
+      <c r="M255" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="256" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A256" t="s">
+        <v>138</v>
+      </c>
+      <c r="B256" t="s">
+        <v>341</v>
+      </c>
+      <c r="C256" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D256" t="s">
+        <v>291</v>
+      </c>
+      <c r="E256" t="s">
+        <v>52</v>
+      </c>
+      <c r="F256" t="s">
+        <v>120</v>
+      </c>
+      <c r="G256" t="s">
+        <v>17</v>
+      </c>
+      <c r="H256" t="s">
+        <v>18</v>
+      </c>
+      <c r="I256" t="s">
+        <v>19</v>
+      </c>
+      <c r="J256" t="s">
+        <v>322</v>
+      </c>
+      <c r="K256" t="s">
+        <v>20</v>
+      </c>
+      <c r="L256" t="s">
+        <v>21</v>
+      </c>
+      <c r="M256" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="257" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A257" t="s">
+        <v>155</v>
+      </c>
+      <c r="B257" t="s">
+        <v>342</v>
+      </c>
+      <c r="C257" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D257" t="s">
+        <v>290</v>
+      </c>
+      <c r="E257" t="s">
+        <v>52</v>
+      </c>
+      <c r="F257" t="s">
+        <v>120</v>
+      </c>
+      <c r="G257" t="s">
+        <v>17</v>
+      </c>
+      <c r="H257" t="s">
+        <v>18</v>
+      </c>
+      <c r="I257" t="s">
+        <v>53</v>
+      </c>
+      <c r="J257" t="s">
+        <v>322</v>
+      </c>
+      <c r="K257" t="s">
+        <v>20</v>
+      </c>
+      <c r="L257" t="s">
+        <v>21</v>
+      </c>
+      <c r="M257" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="258" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A258" t="s">
+        <v>155</v>
+      </c>
+      <c r="B258" t="s">
+        <v>343</v>
+      </c>
+      <c r="C258" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D258" t="s">
+        <v>290</v>
+      </c>
+      <c r="E258" t="s">
+        <v>52</v>
+      </c>
+      <c r="F258" t="s">
+        <v>120</v>
+      </c>
+      <c r="G258" t="s">
+        <v>17</v>
+      </c>
+      <c r="H258" t="s">
+        <v>18</v>
+      </c>
+      <c r="I258" t="s">
+        <v>53</v>
+      </c>
+      <c r="J258" t="s">
+        <v>322</v>
+      </c>
+      <c r="K258" t="s">
+        <v>30</v>
+      </c>
+      <c r="L258" t="s">
+        <v>21</v>
+      </c>
+      <c r="M258" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="259" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A259" t="s">
+        <v>155</v>
+      </c>
+      <c r="B259" t="s">
+        <v>344</v>
+      </c>
+      <c r="C259" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D259" t="s">
+        <v>290</v>
+      </c>
+      <c r="E259" t="s">
+        <v>52</v>
+      </c>
+      <c r="F259" t="s">
+        <v>120</v>
+      </c>
+      <c r="G259" t="s">
+        <v>17</v>
+      </c>
+      <c r="H259" t="s">
+        <v>18</v>
+      </c>
+      <c r="I259" t="s">
+        <v>19</v>
+      </c>
+      <c r="J259" t="s">
+        <v>322</v>
+      </c>
+      <c r="K259" t="s">
+        <v>30</v>
+      </c>
+      <c r="L259" t="s">
+        <v>21</v>
+      </c>
+      <c r="M259" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="260" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A260" t="s">
+        <v>155</v>
+      </c>
+      <c r="B260" t="s">
+        <v>345</v>
+      </c>
+      <c r="C260" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D260" t="s">
+        <v>290</v>
+      </c>
+      <c r="E260" t="s">
+        <v>52</v>
+      </c>
+      <c r="F260" t="s">
+        <v>120</v>
+      </c>
+      <c r="G260" t="s">
+        <v>17</v>
+      </c>
+      <c r="H260" t="s">
+        <v>18</v>
+      </c>
+      <c r="I260" t="s">
+        <v>19</v>
+      </c>
+      <c r="J260" t="s">
+        <v>322</v>
+      </c>
+      <c r="K260" t="s">
+        <v>20</v>
+      </c>
+      <c r="L260" t="s">
+        <v>21</v>
+      </c>
+      <c r="M260" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="261" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A261" t="s">
+        <v>155</v>
+      </c>
+      <c r="B261" t="s">
+        <v>346</v>
+      </c>
+      <c r="C261" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D261" t="s">
+        <v>290</v>
+      </c>
+      <c r="E261" t="s">
+        <v>52</v>
+      </c>
+      <c r="F261" t="s">
+        <v>120</v>
+      </c>
+      <c r="G261" t="s">
+        <v>17</v>
+      </c>
+      <c r="H261" t="s">
+        <v>18</v>
+      </c>
+      <c r="I261" t="s">
+        <v>53</v>
+      </c>
+      <c r="J261" t="s">
+        <v>322</v>
+      </c>
+      <c r="K261" t="s">
+        <v>30</v>
+      </c>
+      <c r="L261" t="s">
+        <v>21</v>
+      </c>
+      <c r="M261" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="262" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A262" t="s">
+        <v>155</v>
+      </c>
+      <c r="B262" t="s">
+        <v>347</v>
+      </c>
+      <c r="C262" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D262" t="s">
+        <v>290</v>
+      </c>
+      <c r="E262" t="s">
+        <v>52</v>
+      </c>
+      <c r="F262" t="s">
+        <v>120</v>
+      </c>
+      <c r="G262" t="s">
+        <v>17</v>
+      </c>
+      <c r="H262" t="s">
+        <v>18</v>
+      </c>
+      <c r="I262" t="s">
+        <v>53</v>
+      </c>
+      <c r="J262" t="s">
+        <v>322</v>
+      </c>
+      <c r="K262" t="s">
+        <v>20</v>
+      </c>
+      <c r="L262" t="s">
+        <v>21</v>
+      </c>
+      <c r="M262" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="263" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A263" t="s">
+        <v>155</v>
+      </c>
+      <c r="B263" t="s">
+        <v>348</v>
+      </c>
+      <c r="C263" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D263" t="s">
+        <v>290</v>
+      </c>
+      <c r="E263" t="s">
+        <v>52</v>
+      </c>
+      <c r="F263" t="s">
+        <v>120</v>
+      </c>
+      <c r="G263" t="s">
+        <v>17</v>
+      </c>
+      <c r="H263" t="s">
+        <v>18</v>
+      </c>
+      <c r="I263" t="s">
+        <v>19</v>
+      </c>
+      <c r="J263" t="s">
+        <v>322</v>
+      </c>
+      <c r="K263" t="s">
+        <v>30</v>
+      </c>
+      <c r="L263" t="s">
+        <v>21</v>
+      </c>
+      <c r="M263" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="264" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A264" t="s">
+        <v>155</v>
+      </c>
+      <c r="B264" t="s">
+        <v>349</v>
+      </c>
+      <c r="C264" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D264" t="s">
+        <v>290</v>
+      </c>
+      <c r="E264" t="s">
+        <v>52</v>
+      </c>
+      <c r="F264" t="s">
+        <v>120</v>
+      </c>
+      <c r="G264" t="s">
+        <v>17</v>
+      </c>
+      <c r="H264" t="s">
+        <v>18</v>
+      </c>
+      <c r="I264" t="s">
+        <v>19</v>
+      </c>
+      <c r="J264" t="s">
+        <v>322</v>
+      </c>
+      <c r="K264" t="s">
+        <v>20</v>
+      </c>
+      <c r="L264" t="s">
+        <v>21</v>
+      </c>
+      <c r="M264" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:M236" xr:uid="{3420B4CD-E5A7-4917-9830-C7287AACEB71}"/>
+  <autoFilter ref="A2:M264" xr:uid="{3420B4CD-E5A7-4917-9830-C7287AACEB71}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:M1"/>
   </mergeCells>
@@ -11727,14 +12974,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA4D436B-8055-44E3-A2FF-23B9BD8F9673}">
-  <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="11.5703125" customWidth="1"/>
-    <col min="3" max="3" width="60.85546875" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" customWidth="1"/>
+    <col min="3" max="3" width="60.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>184</v>
       </c>
@@ -11745,7 +12992,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -11753,7 +13000,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -11764,7 +13011,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -11775,7 +13022,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -11786,7 +13033,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -11797,7 +13044,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B7" s="11">
         <v>45495</v>
       </c>
@@ -11805,7 +13052,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>6</v>
       </c>
@@ -11816,7 +13063,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>7</v>
       </c>
@@ -11827,7 +13074,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>8</v>
       </c>
@@ -11836,6 +13083,25 @@
       </c>
       <c r="C10" t="s">
         <v>302</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11" s="11">
+        <v>45911</v>
+      </c>
+      <c r="C11" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B12" s="11">
+        <v>45911</v>
+      </c>
+      <c r="C12" t="s">
+        <v>353</v>
       </c>
     </row>
   </sheetData>
@@ -11844,50 +13110,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <ProductFamily1 xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
-    <DocType xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3">-</DocType>
-    <AdminPublishingStatus xmlns="d6e223a9-2ed3-49eb-a144-c7920aace86d" xsi:nil="true"/>
-    <AdminComments xmlns="d6e223a9-2ed3-49eb-a144-c7920aace86d" xsi:nil="true"/>
-    <ProductFamily xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3">-</ProductFamily>
-    <ProductLine1 xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
-    <Product1 xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
-    <TypeofDocument xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
-    <BLPublishingStatus xmlns="d6e223a9-2ed3-49eb-a144-c7920aace86d">Not Ready for Publishing</BLPublishingStatus>
-    <RevisionDate xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="c4672b8b-43e2-4139-8cd1-27ad03f081e7" xsi:nil="true"/>
-    <f508be0a0b024b158bf26b5c5377e7cf xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </f508be0a0b024b158bf26b5c5377e7cf>
-    <Product xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3">-</Product>
-    <TypeofRequest xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
-    <qttm xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
-    <DocVersion xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
-    <ProductLine xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3">GPIS</ProductLine>
-    <b301e47fc8e747e89089776eea6c567d xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </b301e47fc8e747e89089776eea6c567d>
-    <BriefDescription xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
-    <KeyProduct_x0028_s_x0029_ xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
-    <DocumentTitle xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007EDDDBC4FB296F4F9CB63BAE8760DE1A" ma:contentTypeVersion="54" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fc9298e5f362f8b2a2f1539074131357">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e6a1524d-d10d-4703-8343-a785c2cc36c3" xmlns:ns3="d6e223a9-2ed3-49eb-a144-c7920aace86d" xmlns:ns4="c4672b8b-43e2-4139-8cd1-27ad03f081e7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4374d41095fb9fe455f76c5bbb6d7977" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="e6a1524d-d10d-4703-8343-a785c2cc36c3"/>
@@ -12396,10 +13618,66 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <ProductFamily1 xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
+    <DocType xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3">-</DocType>
+    <AdminPublishingStatus xmlns="d6e223a9-2ed3-49eb-a144-c7920aace86d" xsi:nil="true"/>
+    <AdminComments xmlns="d6e223a9-2ed3-49eb-a144-c7920aace86d" xsi:nil="true"/>
+    <ProductFamily xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3">-</ProductFamily>
+    <ProductLine1 xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
+    <Product1 xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
+    <TypeofDocument xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
+    <BLPublishingStatus xmlns="d6e223a9-2ed3-49eb-a144-c7920aace86d">Not Ready for Publishing</BLPublishingStatus>
+    <RevisionDate xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="c4672b8b-43e2-4139-8cd1-27ad03f081e7" xsi:nil="true"/>
+    <f508be0a0b024b158bf26b5c5377e7cf xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </f508be0a0b024b158bf26b5c5377e7cf>
+    <Product xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3">-</Product>
+    <TypeofRequest xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
+    <qttm xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
+    <DocVersion xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
+    <ProductLine xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3">GPIS</ProductLine>
+    <b301e47fc8e747e89089776eea6c567d xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </b301e47fc8e747e89089776eea6c567d>
+    <BriefDescription xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
+    <KeyProduct_x0028_s_x0029_ xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
+    <DocumentTitle xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e6a1524d-d10d-4703-8343-a785c2cc36c3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D85D5D23-A9E4-4E12-B1AB-482CBACB0142}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7CD1CAE-1C94-4628-9704-244F487C11F8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e6a1524d-d10d-4703-8343-a785c2cc36c3"/>
+    <ds:schemaRef ds:uri="d6e223a9-2ed3-49eb-a144-c7920aace86d"/>
+    <ds:schemaRef ds:uri="c4672b8b-43e2-4139-8cd1-27ad03f081e7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -12417,21 +13695,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7CD1CAE-1C94-4628-9704-244F487C11F8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D85D5D23-A9E4-4E12-B1AB-482CBACB0142}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e6a1524d-d10d-4703-8343-a785c2cc36c3"/>
-    <ds:schemaRef ds:uri="d6e223a9-2ed3-49eb-a144-c7920aace86d"/>
-    <ds:schemaRef ds:uri="c4672b8b-43e2-4139-8cd1-27ad03f081e7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>